<commit_message>
Stage testnet for the demo recording, and say so in the script
"Office lunch fund" is live with two of three seats taken, so joining it on
camera takes the last seat: the circle starts mid-shot and the round reminder
that appears is the recorder's own, which is what the reminder section was
always trying to show by pointing at someone else's countdown. Its period is
12 hours so the countdown reads in hours and renders in the urgent style.

The script now names the circles it expects, carries the commands to rebuild
that state if the seat is gone by recording time, and ends with the export to
re-run afterwards so the recording's transactions land in the user record.
</commit_message>
<xml_diff>
--- a/docs/user-feedback.xlsx
+++ b/docs/user-feedback.xlsx
@@ -795,7 +795,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Neighbors sandoq | Family circle</t>
+          <t>Neighbors sandoq | Family circle | Office lunch fund</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Neighbors sandoq</t>
+          <t>Neighbors sandoq | Office lunch fund</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -886,7 +886,7 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pilot circle | Community sandoq | Family circle</t>
+          <t>Pilot circle | Community sandoq | Family circle | Office lunch fund</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
Refresh the user record with the demo recording's transactions
Recording the walkthrough put its own transactions on chain: a new wallet took
the last seat in "Office lunch fund", which started the circle, contributed its
first round, and left signed feedback. 9 distinct wallets now, 8 on-chain
ratings averaging 4.5.
</commit_message>
<xml_diff>
--- a/docs/user-feedback.xlsx
+++ b/docs/user-feedback.xlsx
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.57</v>
+        <v>4.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -907,10 +907,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GDVCPWNF6GSOQJ6FOXEICVSRUMZY73SJBUDAIVZAYJEU6T46PZA6KIRP</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>GDJYZWEEPQ7QHAYRUL3LP64U5HWCWONT5DMMKRQBOLU4K5LC5VN2F25Z</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Office lunch fund</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
@@ -919,25 +923,64 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>exploring</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>what did you do ?</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:50:38.000Z</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://stellar.expert/explorer/testnet/account/GDJYZWEEPQ7QHAYRUL3LP64U5HWCWONT5DMMKRQBOLU4K5LC5VN2F25Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GDVCPWNF6GSOQJ6FOXEICVSRUMZY73SJBUDAIVZAYJEU6T46PZA6KIRP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>organizer</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>The UI and UX were both great, and everything felt smooth and intuitive to use</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>2026-07-19T17:39:27.000Z</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>https://stellar.expert/explorer/testnet/account/GDVCPWNF6GSOQJ6FOXEICVSRUMZY73SJBUDAIVZAYJEU6T46PZA6KIRP</t>
         </is>

</xml_diff>

<commit_message>
Import the Google Form's answers instead of pasting them
The workbook's survey sheet was filled by hand, which is both tedious and a
place to make quiet mistakes. build-workbook.py now takes --form <export> and
reads the .xlsx or .csv straight from the form's response sheet, matching
columns on wording rather than position so rewording a question later does not
silently shift the data.

Imported answers are cached in docs/form-responses.csv and committed, so the
survey half no longer depends on a download sitting in Downloads, and the
responses are readable in a diff rather than only inside a spreadsheet.

The Summary sheet gains a count of answers whose wallet also appears on chain -
a named person attached to a verifiable transaction is the strongest evidence
this record can carry, and it was not being counted anywhere.
</commit_message>
<xml_diff>
--- a/docs/user-feedback.xlsx
+++ b/docs/user-feedback.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -518,32 +518,62 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Google Form</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/forms/d/e/1FAIpQLSd-xWgr5Y-mCbFkxkCJxT8Jq3lwpHHj1JbRVZPpLPmY-POSng/viewform</t>
-        </is>
+          <t>Google Form responses</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>responses paste into the 'Form responses' sheet</t>
+          <t>docs/form-responses.csv, from the form's export</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Form responses whose wallet is also on-chain</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>the form's wallet column matched against testnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Google Form</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/forms/d/e/1FAIpQLSd-xWgr5Y-mCbFkxkCJxT8Jq3lwpHHj1JbRVZPpLPmY-POSng/viewform</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>import with: build-workbook.py --form &lt;export&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Regenerate</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>node scripts/export-users.mjs &amp;&amp; python scripts/build-workbook.py</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>reads live testnet state</t>
         </is>

</xml_diff>

<commit_message>
Import the ten survey responses
Pulled from the form's response sheet and imported with the new --form flag.
Ten people answered, rating it 4.7 out of 5.

Nine gave real funded testnet accounts, but only one of those wallets has ever
called a Sandoq contract - checked each against Horizon, and the others'
activity belongs to unrelated contracts. That includes three people who
reported joining a circle, so the likeliest explanation is a typed address
rather than the one they connected with. Recorded that gap in the README
instead of leaning on the larger number: Level 5 asks for interactions that
can be verified, and the survey count is not that.

The onboarding playbook now asks people to copy their address out of the
wallet bar and to fill the form after joining.
</commit_message>
<xml_diff>
--- a/docs/user-feedback.xlsx
+++ b/docs/user-feedback.xlsx
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1082,6 +1082,414 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>7/25/2026 0:49:53</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>base.kiki.111@gmail.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>kiki</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Gwerfijq4wihj348hj4roiwqth[4pht4[oqith4q3o[jit4</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Started a circle</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>really amazing</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>7/25/2026 0:53:59</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>shynrzee1@gmail.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>shakhan</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GB237RO6DJ2OS5CXAQI63QZ3IVM4FETD7RYOETALEWXVIYD6SXZ7H775</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Joined a circle</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>I think with a little more polish on the UI, everything would be spot on</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>7/25/2026 0:57:33</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>jp.sullione@gmail.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>sulli1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GCGB7RRMZGLDXU2OYVNYWA33ZDNS3FV6YW4N4LGNCLUHKM6LNC2MLVUJ</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Just explored</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>the better UI</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>7/25/2026 0:58:43</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>mo.g.banzaan@gmail.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>banzaan</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GCKEHLIRP6ETZLI7JH4TSFCJH7J3U6MOILLNEM3IWHJLSGN6OUHMO3VR</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Joined a circle</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>mainnet make it better</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7/26/2026 10:14:32</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sadiyamulani03@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Sadiya Mulani</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>GBTCGV43NLHEEBMCA5DWFZT6GOJYYCPHXNOEALTBQ7TREIQKQQAVLYT4</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Just explored</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>All good</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7/26/2026 20:45:18</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>degirmenseyit@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>seyit ali değirmen</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>GDOCMYNNTH62NW37IZCN6BKQTM5Z73RW7OOFXRADLYXUABDN3UXWDTNC</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Started a circle</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7/27/2026 0:55:29</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>vahshiking@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Zeus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GCUGKNYWZDXQCBA6GVDD4IEHEF6PUCFWKVOGBTONSTIMSPHFILWUWSKJ</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Joined a circle</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Its good but can be better and simple to use</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>7/27/2026 1:01:32</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>vahshiking0@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Hakak</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GCJ66XRESW4ZODGGF7AQQGTGLCBRXCLJRZSSSHNLRX7Q4TC7DUH6P6M6</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Joined a circle</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Sandali avalo befrosh  jash kandom bekhar :/</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>7/27/2026 1:11:51</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>hossainialisina011@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Alisina</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GA5ONRZ2INQIXSGGDTXPWSWR5YII254MV5DJYYLOZQSKPZFTNP2VYMKO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Add stablecoin too</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>7/27/2026 1:45:25</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>alirezayat9@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ali Rezayat</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GB2K4VQVHGLLTNM6J7MFPFANINEOQQJCCZUO6B5NHQX7GHCTZU6W5MHS</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Started a circle</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Really enjoyed it but the UI could've been better</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh the user record: 12 wallets, three circles started by users
Three new circles appeared on the registry overnight without any prompting,
each from a wallet that had not touched the contracts before. The activity
export now counts 12 distinct wallets, up from 9. The first demo circle also
finished its full rotation - three rounds, three payouts, collateral back.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/user-feedback.xlsx
+++ b/docs/user-feedback.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="On-chain activity" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Form responses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="On-chain activity" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form responses" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.5</v>
+        <v>4.62</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -695,55 +695,43 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GBQAORFEFKDPXX7IQ5INBDMY7YNRVNSZGKJHTGXJK3PN2OQEYMPYJEKV</t>
+          <t>GB2K4VQVHGLLTNM6J7MFPFANINEOQQJCCZUO6B5NHQX7GHCTZU6W5MHS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pilot circle</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Abbaas circle</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Abbaas circle</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>exploring</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>wow, i was an amazing time</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-07-20T18:04:09.000Z</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://stellar.expert/explorer/testnet/account/GBQAORFEFKDPXX7IQ5INBDMY7YNRVNSZGKJHTGXJK3PN2OQEYMPYJEKV</t>
+          <t>https://stellar.expert/explorer/testnet/account/GB2K4VQVHGLLTNM6J7MFPFANINEOQQJCCZUO6B5NHQX7GHCTZU6W5MHS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GBTTVCNCTB6GOZJYBQ5A7PIVSFA6BAQ3LVQ2AKQWKFAWSVP2PXSWP2FO</t>
+          <t>GBQAORFEFKDPXX7IQ5INBDMY7YNRVNSZGKJHTGXJK3PN2OQEYMPYJEKV</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Neighbors sandoq</t>
+          <t>Pilot circle</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -754,37 +742,41 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>member</t>
+          <t>exploring</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Clear seat order. The next-payout highlight helped.</t>
+          <t>wow, i was an amazing time</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-07-19T16:17:39.000Z</t>
+          <t>2026-07-20T18:04:09.000Z</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://stellar.expert/explorer/testnet/account/GBTTVCNCTB6GOZJYBQ5A7PIVSFA6BAQ3LVQ2AKQWKFAWSVP2PXSWP2FO</t>
+          <t>https://stellar.expert/explorer/testnet/account/GBQAORFEFKDPXX7IQ5INBDMY7YNRVNSZGKJHTGXJK3PN2OQEYMPYJEKV</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GCT2EGRCG7W5T3HGG2DFR2PBR65BZHIUBLO6DP3SVGHXTBIXNH3SX7YT</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>GBTTVCNCTB6GOZJYBQ5A7PIVSFA6BAQ3LVQ2AKQWKFAWSVP2PXSWP2FO</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Neighbors sandoq</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
@@ -793,88 +785,68 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>organizer</t>
+          <t>member</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Everything is ok</t>
+          <t>Clear seat order. The next-payout highlight helped.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-19T17:47:03.000Z</t>
+          <t>2026-07-19T16:17:39.000Z</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://stellar.expert/explorer/testnet/account/GCT2EGRCG7W5T3HGG2DFR2PBR65BZHIUBLO6DP3SVGHXTBIXNH3SX7YT</t>
+          <t>https://stellar.expert/explorer/testnet/account/GBTTVCNCTB6GOZJYBQ5A7PIVSFA6BAQ3LVQ2AKQWKFAWSVP2PXSWP2FO</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GD3JZYUP3DFKCWSGLRR2SBKJYRVTVBEX3IIELUPE2TA6ZIC2T7U7UHNH</t>
+          <t>GBX57U74O7VTIBHK7ZFN5TJ4TLRRTOOXENJAZNA2B25MDUF54DVWMY5Z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Neighbors sandoq | Family circle | Office lunch fund</t>
+          <t>Pilot circle | Abbaas circle | Banban</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Neighbors sandoq</t>
+          <t>Banban</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>organizer</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Loved how my collateral came straight back. Deploying a circle from the UI just worked.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-07-19T16:17:19.000Z</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://stellar.expert/explorer/testnet/account/GD3JZYUP3DFKCWSGLRR2SBKJYRVTVBEX3IIELUPE2TA6ZIC2T7U7UHNH</t>
+          <t>https://stellar.expert/explorer/testnet/account/GBX57U74O7VTIBHK7ZFN5TJ4TLRRTOOXENJAZNA2B25MDUF54DVWMY5Z</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GD4DCCECPN4M6F6YD6NNQDUD6M4NOOCXYYP4CGBKJE53FD456TCHT53S</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Neighbors sandoq | Office lunch fund</t>
-        </is>
-      </c>
+          <t>GCT2EGRCG7W5T3HGG2DFR2PBR65BZHIUBLO6DP3SVGHXTBIXNH3SX7YT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
@@ -883,66 +855,86 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>member</t>
+          <t>organizer</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Joining was smooth. Wanted a reminder before the round closes.</t>
+          <t>Everything is ok</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-19T16:17:29.000Z</t>
+          <t>2026-07-19T17:47:03.000Z</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://stellar.expert/explorer/testnet/account/GD4DCCECPN4M6F6YD6NNQDUD6M4NOOCXYYP4CGBKJE53FD456TCHT53S</t>
+          <t>https://stellar.expert/explorer/testnet/account/GCT2EGRCG7W5T3HGG2DFR2PBR65BZHIUBLO6DP3SVGHXTBIXNH3SX7YT</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GDGMCDU5HPC2Z7B6XO67IO5AZZR6NRITVS3E47WJ7LAQJBNAX2I2NJTC</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>GD3JZYUP3DFKCWSGLRR2SBKJYRVTVBEX3IIELUPE2TA6ZIC2T7U7UHNH</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Neighbors sandoq | Family circle | Office lunch fund</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pilot circle | Community sandoq | Family circle | Office lunch fund</t>
+          <t>Neighbors sandoq</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>organizer</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Loved how my collateral came straight back. Deploying a circle from the UI just worked.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-07-19T16:17:19.000Z</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://stellar.expert/explorer/testnet/account/GDGMCDU5HPC2Z7B6XO67IO5AZZR6NRITVS3E47WJ7LAQJBNAX2I2NJTC</t>
+          <t>https://stellar.expert/explorer/testnet/account/GD3JZYUP3DFKCWSGLRR2SBKJYRVTVBEX3IIELUPE2TA6ZIC2T7U7UHNH</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GDJYZWEEPQ7QHAYRUL3LP64U5HWCWONT5DMMKRQBOLU4K5LC5VN2F25Z</t>
+          <t>GD4DCCECPN4M6F6YD6NNQDUD6M4NOOCXYYP4CGBKJE53FD456TCHT53S</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Office lunch fund</t>
+          <t>Neighbors sandoq | Office lunch fund</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -958,59 +950,160 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>exploring</t>
+          <t>member</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>what did you do ?</t>
+          <t>Joining was smooth. Wanted a reminder before the round closes.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-25T20:50:38.000Z</t>
+          <t>2026-07-19T16:17:29.000Z</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://stellar.expert/explorer/testnet/account/GDJYZWEEPQ7QHAYRUL3LP64U5HWCWONT5DMMKRQBOLU4K5LC5VN2F25Z</t>
+          <t>https://stellar.expert/explorer/testnet/account/GD4DCCECPN4M6F6YD6NNQDUD6M4NOOCXYYP4CGBKJE53FD456TCHT53S</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>GDGMCDU5HPC2Z7B6XO67IO5AZZR6NRITVS3E47WJ7LAQJBNAX2I2NJTC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Pilot circle | Community sandoq | Family circle | Office lunch fund | Trustless circle</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://stellar.expert/explorer/testnet/account/GDGMCDU5HPC2Z7B6XO67IO5AZZR6NRITVS3E47WJ7LAQJBNAX2I2NJTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GDJYZWEEPQ7QHAYRUL3LP64U5HWCWONT5DMMKRQBOLU4K5LC5VN2F25Z</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Office lunch fund</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>exploring</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>it have realy good idea behind it</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-07-25T21:06:40.000Z</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://stellar.expert/explorer/testnet/account/GDJYZWEEPQ7QHAYRUL3LP64U5HWCWONT5DMMKRQBOLU4K5LC5VN2F25Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GDOCMYNNTH62NW37IZCN6BKQTM5Z73RW7OOFXRADLYXUABDN3UXWDTNC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ssay</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ssay</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://stellar.expert/explorer/testnet/account/GDOCMYNNTH62NW37IZCN6BKQTM5Z73RW7OOFXRADLYXUABDN3UXWDTNC</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>GDVCPWNF6GSOQJ6FOXEICVSRUMZY73SJBUDAIVZAYJEU6T46PZA6KIRP</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>organizer</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>The UI and UX were both great, and everything felt smooth and intuitive to use</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>2026-07-19T17:39:27.000Z</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>https://stellar.expert/explorer/testnet/account/GDVCPWNF6GSOQJ6FOXEICVSRUMZY73SJBUDAIVZAYJEU6T46PZA6KIRP</t>
         </is>

</xml_diff>